<commit_message>
Exclude Zamorano and Munk from spine capacity counts per practice direction
Both stay on the Physician Roster tab for reference (each appears on the
Sept 7 ASC/clinic schedule) under an explicit "NOT Counted Toward Spine
Capacity" section. Counted spine surgeons 6 -> 4 (Varghese, Salar, Maslak,
McCarty), spine-capable total 10 -> 8, counted spine new-patient YTD
1,424 -> 1,260. Start Here who-is-counted guidance updated to match.
Recalculated clean: 357 formulas, zero errors.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MP7PpTPreNsinr43dcL1GA
</commit_message>
<xml_diff>
--- a/pm/Clinic_Capacity_Audit.xlsx
+++ b/pm/Clinic_Capacity_Audit.xlsx
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="182">
   <si>
     <t xml:space="preserve">Clinic Capacity Audit | Start Here</t>
   </si>
@@ -159,13 +159,13 @@
     <t xml:space="preserve">Who Is Counted</t>
   </si>
   <si>
-    <t xml:space="preserve">Clinic-day counts cover the physicians on the Physician Roster tab (Ortho &amp; Spine only). The Ortho count covers the 7 Ortho surgeons; "Ortho Physicians Out" means how many of those 7 are out - enter 0 when everyone is available (blank is treated as 0). The roster lists spine surgeons and interventional pain physicians separately so the same inclusion rule is applied every week. Three names on the Sept 7 schedule are pending confirmation - see the roster tab.</t>
+    <t xml:space="preserve">Clinic-day counts cover the physicians on the Physician Roster tab (Ortho &amp; Spine only): 4 spine surgeons + 4 interventional pain physicians, and 7 Ortho surgeons. Zamorano and Munk appear on the roster for reference but are NOT counted toward Spine capacity (practice direction). "Ortho Physicians Out" means how many of the 7 Ortho surgeons are out - enter 0 when everyone is available (blank is treated as 0). Three names on the Sept 7 schedule are pending confirmation - see the roster tab.</t>
   </si>
   <si>
     <t xml:space="preserve">Physician Roster | Ortho &amp; Spine</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference roster for this audit - Ortho and Spine service lines only. The Weekly Audit clinic-day counts and "Ortho Physicians Out" refer to the physicians below.</t>
+    <t xml:space="preserve">Reference roster for this audit - Ortho and Spine service lines only. The Weekly Audit clinic-day counts and "Ortho Physicians Out" refer to the physicians below. Zamorano and Munk are listed for reference and are NOT counted toward Spine capacity.</t>
   </si>
   <si>
     <t xml:space="preserve">Physician</t>
@@ -192,7 +192,7 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">SPINE - Surgeons</t>
+    <t xml:space="preserve">SPINE - Surgeons (counted toward Spine capacity)</t>
   </si>
   <si>
     <t xml:space="preserve">Jeffrey Varghese</t>
@@ -243,9 +243,120 @@
     <t xml:space="preserve">Highest spine new-patient volume YTD.</t>
   </si>
   <si>
+    <t xml:space="preserve">SPINE - Interventional Pain (non-surgical spine)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anthony J. Oddo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spine Pain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Director of Pain Management - spine pain, injections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Oddo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kevin R. Lee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pain management + functional neurosurgery - minimally invasive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K Lee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brian Kassa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fellowship-trained pain management - spine &amp; joint interventions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B Kassa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hanish Singh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pain management - spine diagnostics, injections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H Singh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORTHO - Surgeons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeffrey Mendelson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ortho Surgeon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chief of Orthopedic Surgery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">David Mendelson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fellowship-trained orthopedic surgeon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stephen Mendelson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orthopedic surgeon (fellowship-trained, Israel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alice Mendelson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Women's bone health, fracture prevention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preetinder Bhullar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hip &amp; knee replacement (arthroplasty)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bhullar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ben Mayo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sports medicine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mayo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joseph Yacisen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sports medicine (25+ yrs; military service)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yacisen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harbor Beach weeks 2 &amp; 4 (per schedule note).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On the Sept 7 Schedule - NOT Counted Toward Spine Capacity (practice direction, Aug 2026)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lucia Zamorano</t>
   </si>
   <si>
+    <t xml:space="preserve">Spine (not counted)</t>
+  </si>
+  <si>
     <t xml:space="preserve">MD, FAANOS, FICS</t>
   </si>
   <si>
@@ -255,7 +366,7 @@
     <t xml:space="preserve">L Zamorano / "Dr. Zam."</t>
   </si>
   <si>
-    <t xml:space="preserve">Troy clinics Mon &amp; Thu; 1st Monday of month blocked at hospital (per schedule note).</t>
+    <t xml:space="preserve">Not counted toward Spine capacity per practice direction. Troy clinics Mon &amp; Thu; 1st Monday of month blocked at hospital (per schedule note).</t>
   </si>
   <si>
     <t xml:space="preserve">A. Munk</t>
@@ -267,130 +378,25 @@
     <t xml:space="preserve">A Munk</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm listing/role with practice - appears in internal data and on the schedule, not on the website provider pages.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SPINE - Interventional Pain (non-surgical spine)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anthony J. Oddo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spine Pain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Director of Pain Management - spine pain, injections</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Oddo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kevin R. Lee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pain management + functional neurosurgery - minimally invasive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K Lee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brian Kassa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fellowship-trained pain management - spine &amp; joint interventions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B Kassa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hanish Singh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pain management - spine diagnostics, injections</t>
-  </si>
-  <si>
-    <t xml:space="preserve">H Singh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ORTHO - Surgeons</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jeffrey Mendelson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ortho Surgeon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chief of Orthopedic Surgery</t>
-  </si>
-  <si>
-    <t xml:space="preserve">David Mendelson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fellowship-trained orthopedic surgeon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stephen Mendelson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Orthopedic surgeon (fellowship-trained, Israel)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alice Mendelson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Women's bone health, fracture prevention</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preetinder Bhullar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hip &amp; knee replacement (arthroplasty)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bhullar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ben Mayo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sports medicine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mayo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joseph Yacisen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sports medicine (25+ yrs; military service)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yacisen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harbor Beach weeks 2 &amp; 4 (per schedule note).</t>
+    <t xml:space="preserve">Not counted toward Spine capacity per practice direction. Appears in internal data and on the schedule, not on the website provider pages.</t>
   </si>
   <si>
     <t xml:space="preserve">Roster Counts</t>
   </si>
   <si>
-    <t xml:space="preserve">Spine surgeons</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Counts the roster rows above by Service Line.</t>
+    <t xml:space="preserve">Spine surgeons (counted)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counts the roster rows above by Service Line. Excludes Zamorano and Munk per practice direction.</t>
   </si>
   <si>
     <t xml:space="preserve">Spine interventional pain physicians</t>
   </si>
   <si>
-    <t xml:space="preserve">Spine-capable physicians (total)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roster doc cites 9 (A. Munk pending confirmation with the practice); 10 if confirmed.</t>
+    <t xml:space="preserve">Spine-capable physicians (counted total)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zamorano and Munk excluded; with them the schedule shows 10 spine-capable physicians.</t>
   </si>
   <si>
     <t xml:space="preserve">Ortho surgeons</t>
@@ -399,10 +405,10 @@
     <t xml:space="preserve">Matches the Start Here assumption: 16 required days = full 7-surgeon roster available.</t>
   </si>
   <si>
-    <t xml:space="preserve">Spine new patients | Jan 1 - Jul 15, 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Internal new-patient data via the roster doc. Volume does not equal conversion.</t>
+    <t xml:space="preserve">Spine new patients | Jan 1 - Jul 15, 2026 (counted surgeons)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Internal new-patient data via the roster doc; excludes Zamorano (51) and Munk (113). Volume does not equal conversion.</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm With Practice Before Treating This Roster as Final</t>
@@ -420,7 +426,7 @@
     <t xml:space="preserve">Sources</t>
   </si>
   <si>
-    <t xml:space="preserve">Physicians: brand/provider-roster-by-service-line.md (synergyhealth.org /providers/ crawl + page metadata, July 15, 2026) - Ortho and Spine service lines only, as requested. Schedule cross-check: ASC_Clinic_Schedule_Sept_7th.xlsx ("Clinic and ASC Schedule" and "Proposed" tabs) - every physician listed above appears on that schedule. Spine new-patient counts: internal new-patient data, Jan 1 - Jul 15, 2026, via the same roster doc. Hand, foot &amp; ankle, primary care, PT/OT, and PA staff are intentionally excluded.</t>
+    <t xml:space="preserve">Physicians: brand/provider-roster-by-service-line.md (synergyhealth.org /providers/ crawl + page metadata, July 15, 2026) - Ortho and Spine service lines only, as requested. Schedule cross-check: ASC_Clinic_Schedule_Sept_7th.xlsx ("Clinic and ASC Schedule" and "Proposed" tabs) - every physician listed above appears on that schedule. Spine new-patient counts: internal new-patient data, Jan 1 - Jul 15, 2026, via the same roster doc. Zamorano and Munk excluded from spine counts per practice direction (Aug 11, 2026). Hand, foot &amp; ankle, primary care, PT/OT, and PA staff are intentionally excluded.</t>
   </si>
   <si>
     <t xml:space="preserve">16-Week Clinic Capacity Audit</t>
@@ -2074,8 +2080,8 @@
     <tabColor rgb="FF0E7490"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
-  <sheetFormatPr defaultColWidth="10.76953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H41"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
@@ -2247,354 +2253,349 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="s">
+    <row r="10" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="C10" s="24" t="s">
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="B11" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="E10" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="F10" s="24" t="s">
+      <c r="C11" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="G10" s="26" t="n">
-        <v>51</v>
-      </c>
-      <c r="H10" s="25" t="s">
+      <c r="D11" s="25" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="25" t="s">
-        <v>67</v>
       </c>
       <c r="E11" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F11" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="G11" s="26"/>
+      <c r="H11" s="25"/>
+    </row>
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="G11" s="26" t="n">
-        <v>113</v>
-      </c>
-      <c r="H11" s="25" t="s">
+      <c r="E12" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="24" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="25"/>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="25" t="s">
         <v>71</v>
-      </c>
-      <c r="B13" s="24" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="D13" s="25" t="s">
-        <v>74</v>
       </c>
       <c r="E13" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="G13" s="26"/>
       <c r="H13" s="25"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>47</v>
       </c>
       <c r="D14" s="25" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E14" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="G14" s="26"/>
       <c r="H14" s="25"/>
     </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" s="24" t="s">
-        <v>72</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="D15" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="E15" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="F15" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="G15" s="26"/>
-      <c r="H15" s="25"/>
+    <row r="15" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>47</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E16" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="G16" s="26"/>
       <c r="H16" s="25"/>
     </row>
-    <row r="17" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="F17" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17" s="26"/>
+      <c r="H17" s="25"/>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C18" s="24" t="s">
         <v>47</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="E18" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="G18" s="26"/>
       <c r="H18" s="25"/>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C19" s="24" t="s">
         <v>47</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="E19" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="G19" s="26"/>
       <c r="H19" s="25"/>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C20" s="24" t="s">
         <v>47</v>
       </c>
       <c r="D20" s="25" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E20" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G20" s="26"/>
       <c r="H20" s="25"/>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>47</v>
       </c>
       <c r="D21" s="25" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E21" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F21" s="24" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G21" s="26"/>
       <c r="H21" s="25"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="23" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C22" s="24" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="D22" s="25" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E22" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F22" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="G22" s="26"/>
+      <c r="H22" s="25" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+    </row>
+    <row r="24" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="G22" s="26"/>
-      <c r="H22" s="25"/>
-    </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="s">
+      <c r="B24" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="B23" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="C23" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="D23" s="25" t="s">
+      <c r="C24" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="E23" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="F23" s="24" t="s">
+      <c r="D24" s="25" t="s">
         <v>100</v>
-      </c>
-      <c r="G23" s="26"/>
-      <c r="H23" s="25"/>
-    </row>
-    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="B24" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="C24" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="D24" s="25" t="s">
-        <v>102</v>
       </c>
       <c r="E24" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F24" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="G24" s="26" t="n">
+        <v>51</v>
+      </c>
+      <c r="H24" s="25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="G24" s="26"/>
-      <c r="H24" s="25" t="s">
+      <c r="B25" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="C25" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="E25" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="F25" s="24" t="s">
         <v>105</v>
       </c>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-    </row>
-    <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="27" t="s">
+      <c r="G25" s="26" t="n">
+        <v>113</v>
+      </c>
+      <c r="H25" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="B27" s="27"/>
-      <c r="C27" s="28" t="n">
-        <f aca="false">COUNTIF($B$6:$B$24,"Spine Surgeon")</f>
-        <v>6</v>
-      </c>
-      <c r="D27" s="29" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
     </row>
     <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="27" t="s">
@@ -2602,10 +2603,12 @@
       </c>
       <c r="B28" s="27"/>
       <c r="C28" s="28" t="n">
-        <f aca="false">COUNTIF($B$6:$B$24,"Spine Pain")</f>
+        <f aca="false">COUNTIF($B$6:$B$25,"Spine Surgeon")</f>
         <v>4</v>
       </c>
-      <c r="D28" s="29"/>
+      <c r="D28" s="29" t="s">
+        <v>109</v>
+      </c>
       <c r="E28" s="29"/>
       <c r="F28" s="29"/>
       <c r="G28" s="29"/>
@@ -2613,16 +2616,14 @@
     </row>
     <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="27" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B29" s="27"/>
       <c r="C29" s="28" t="n">
-        <f aca="false">C27+C28</f>
-        <v>10</v>
-      </c>
-      <c r="D29" s="29" t="s">
-        <v>110</v>
-      </c>
+        <f aca="false">COUNTIF($B$6:$B$25,"Spine Pain")</f>
+        <v>4</v>
+      </c>
+      <c r="D29" s="29"/>
       <c r="E29" s="29"/>
       <c r="F29" s="29"/>
       <c r="G29" s="29"/>
@@ -2634,8 +2635,8 @@
       </c>
       <c r="B30" s="27"/>
       <c r="C30" s="28" t="n">
-        <f aca="false">COUNTIF($B$6:$B$24,"Ortho Surgeon")</f>
-        <v>7</v>
+        <f aca="false">C28+C29</f>
+        <v>8</v>
       </c>
       <c r="D30" s="29" t="s">
         <v>112</v>
@@ -2651,8 +2652,8 @@
       </c>
       <c r="B31" s="27"/>
       <c r="C31" s="28" t="n">
-        <f aca="false">SUM($G$6:$G$11)</f>
-        <v>1424</v>
+        <f aca="false">COUNTIF($B$6:$B$25,"Ortho Surgeon")</f>
+        <v>7</v>
       </c>
       <c r="D31" s="29" t="s">
         <v>114</v>
@@ -2662,33 +2663,38 @@
       <c r="G31" s="29"/>
       <c r="H31" s="29"/>
     </row>
-    <row r="33" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+    <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-    </row>
-    <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="30" t="s">
+      <c r="B32" s="27"/>
+      <c r="C32" s="28" t="n">
+        <f aca="false">SUM($G$6:$G$9)</f>
+        <v>1260</v>
+      </c>
+      <c r="D32" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="B34" s="30"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30"/>
-      <c r="F34" s="30"/>
-      <c r="G34" s="30"/>
-      <c r="H34" s="30"/>
+      <c r="E32" s="29"/>
+      <c r="F32" s="29"/>
+      <c r="G32" s="29"/>
+      <c r="H32" s="29"/>
+    </row>
+    <row r="34" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="30" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B35" s="30"/>
       <c r="C35" s="30"/>
@@ -2700,7 +2706,7 @@
     </row>
     <row r="36" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="30" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B36" s="30"/>
       <c r="C36" s="30"/>
@@ -2710,32 +2716,34 @@
       <c r="G36" s="30"/>
       <c r="H36" s="30"/>
     </row>
-    <row r="38" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
-    </row>
-    <row r="39" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
+    <row r="37" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
+      <c r="B37" s="30"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="30"/>
+      <c r="E37" s="30"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="30"/>
+      <c r="H37" s="30"/>
+    </row>
+    <row r="39" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2"/>
+      <c r="A40" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -2744,16 +2752,25 @@
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
     </row>
+    <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="23">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A26:H26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="D27:H27"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A27:H27"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="D28:H28"/>
     <mergeCell ref="A29:B29"/>
@@ -2762,16 +2779,18 @@
     <mergeCell ref="D30:H30"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="D31:H31"/>
-    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="D32:H32"/>
     <mergeCell ref="A34:H34"/>
     <mergeCell ref="A35:H35"/>
     <mergeCell ref="A36:H36"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A39:H40"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A40:H41"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2815,7 +2834,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2842,7 +2861,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="31" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B2" s="31"/>
       <c r="C2" s="31"/>
@@ -2894,7 +2913,7 @@
     </row>
     <row r="4" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -2904,7 +2923,7 @@
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -2912,13 +2931,13 @@
       <c r="M4" s="4"/>
       <c r="N4" s="4"/>
       <c r="O4" s="4" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
       <c r="R4" s="4"/>
       <c r="S4" s="4" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="T4" s="4"/>
       <c r="U4" s="4"/>
@@ -2952,73 +2971,73 @@
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G6" s="33" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H6" s="33" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I6" s="33" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J6" s="33" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="K6" s="33" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="L6" s="33" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="M6" s="33" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="N6" s="33" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="O6" s="33" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="P6" s="33" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Q6" s="33" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="R6" s="33" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="S6" s="33" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="T6" s="33" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="U6" s="33" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="V6" s="33" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="W6" s="33" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3029,7 +3048,7 @@
         <v>46244</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D7" s="36"/>
       <c r="E7" s="36"/>
@@ -3087,7 +3106,7 @@
         <v>46251</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D8" s="43"/>
       <c r="E8" s="43"/>
@@ -3145,7 +3164,7 @@
         <v>46258</v>
       </c>
       <c r="C9" s="41" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D9" s="43"/>
       <c r="E9" s="43"/>
@@ -3203,7 +3222,7 @@
         <v>46265</v>
       </c>
       <c r="C10" s="41" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D10" s="43"/>
       <c r="E10" s="43"/>
@@ -3261,7 +3280,7 @@
         <v>46272</v>
       </c>
       <c r="C11" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D11" s="43"/>
       <c r="E11" s="43"/>
@@ -3319,7 +3338,7 @@
         <v>46279</v>
       </c>
       <c r="C12" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D12" s="43"/>
       <c r="E12" s="43"/>
@@ -3377,7 +3396,7 @@
         <v>46286</v>
       </c>
       <c r="C13" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D13" s="43"/>
       <c r="E13" s="43"/>
@@ -3435,7 +3454,7 @@
         <v>46293</v>
       </c>
       <c r="C14" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D14" s="43"/>
       <c r="E14" s="43"/>
@@ -3493,7 +3512,7 @@
         <v>46300</v>
       </c>
       <c r="C15" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D15" s="43"/>
       <c r="E15" s="43"/>
@@ -3551,7 +3570,7 @@
         <v>46307</v>
       </c>
       <c r="C16" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D16" s="43"/>
       <c r="E16" s="43"/>
@@ -3609,7 +3628,7 @@
         <v>46314</v>
       </c>
       <c r="C17" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D17" s="43"/>
       <c r="E17" s="43"/>
@@ -3667,7 +3686,7 @@
         <v>46321</v>
       </c>
       <c r="C18" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D18" s="43"/>
       <c r="E18" s="43"/>
@@ -3725,7 +3744,7 @@
         <v>46328</v>
       </c>
       <c r="C19" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D19" s="43"/>
       <c r="E19" s="43"/>
@@ -3783,7 +3802,7 @@
         <v>46335</v>
       </c>
       <c r="C20" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D20" s="43"/>
       <c r="E20" s="43"/>
@@ -3841,7 +3860,7 @@
         <v>46342</v>
       </c>
       <c r="C21" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D21" s="43"/>
       <c r="E21" s="43"/>
@@ -3899,7 +3918,7 @@
         <v>46349</v>
       </c>
       <c r="C22" s="48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D22" s="43"/>
       <c r="E22" s="43"/>
@@ -4162,7 +4181,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4176,7 +4195,7 @@
     </row>
     <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4202,7 +4221,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="50" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B4" s="50"/>
       <c r="C4" s="50"/>
@@ -4228,34 +4247,34 @@
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B6" s="33" t="s">
         <v>37</v>
       </c>
       <c r="C6" s="33" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D6" s="33" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E6" s="33" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F6" s="33" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G6" s="33" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H6" s="33" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="I6" s="33" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="J6" s="33" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4846,7 +4865,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4858,7 +4877,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="55" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B2" s="55"/>
       <c r="C2" s="55"/>
@@ -4880,28 +4899,28 @@
     </row>
     <row r="4" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F4" s="33" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G4" s="33" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="H4" s="33" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4950,7 +4969,7 @@
     </row>
     <row r="7" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
@@ -4962,28 +4981,28 @@
     </row>
     <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C8" s="33" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D8" s="33" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G8" s="33" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H8" s="33" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5532,7 +5551,7 @@
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="70" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B25" s="70"/>
       <c r="C25" s="70"/>
@@ -5544,7 +5563,7 @@
     </row>
     <row r="26" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -5556,7 +5575,7 @@
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B27" s="9"/>
       <c r="C27" s="9"/>

</xml_diff>